<commit_message>
Back to round 1
</commit_message>
<xml_diff>
--- a/QuizSettings.xlsx
+++ b/QuizSettings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cafnzholding-my.sharepoint.com/personal/thom_van_dusschoten_synerlogic_nl/Documents/Documenten/GitHub/Sustainability-quiz-TEST/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{6C329D2D-B3E9-4563-A84D-2DB2372B69CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{738D2597-F743-433C-9301-7D009E531646}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{6C329D2D-B3E9-4563-A84D-2DB2372B69CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E38F0171-88A6-4784-961F-63B8F602B60E}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -473,7 +473,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">

</xml_diff>